<commit_message>
complete version with s/n customer p/n and cust rev etc
</commit_message>
<xml_diff>
--- a/examples/TAAT/ใบสั่งงาน TAAT.xlsx
+++ b/examples/TAAT/ใบสั่งงาน TAAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vatska\software\examples\TAAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17C9108-E61C-4C85-A699-1E624C8B9206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43BB9E59-8546-4012-89BB-A00488E44987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{874D8AF1-DF56-4DEE-86B1-A5E2F5D42D71}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="135">
   <si>
     <r>
       <t>บริษัท แวตสก้า จำกัด/ Vatska Company Limited</t>
@@ -487,9 +487,6 @@
   </si>
   <si>
     <t>What if " LMT55, Pharmed or E3603" then show dropdown list" worksheet A2, column D,E,F -line 38-48</t>
-  </si>
-  <si>
-    <t>LMT_55</t>
   </si>
 </sst>
 </file>
@@ -1151,7 +1148,58 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1160,61 +1208,10 @@
     <xf numFmtId="164" fontId="15" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1739,7 +1736,7 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>685804</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>324768</xdr:rowOff>
+      <xdr:rowOff>320958</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1781,7 +1778,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>701040</xdr:colOff>
+      <xdr:colOff>704850</xdr:colOff>
       <xdr:row>42</xdr:row>
       <xdr:rowOff>932</xdr:rowOff>
     </xdr:to>
@@ -1825,9 +1822,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>708133</xdr:colOff>
+      <xdr:colOff>704323</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>286703</xdr:rowOff>
+      <xdr:rowOff>282893</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1869,9 +1866,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>701992</xdr:colOff>
+      <xdr:colOff>705802</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>287839</xdr:rowOff>
+      <xdr:rowOff>284029</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1913,7 +1910,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>704850</xdr:colOff>
+      <xdr:colOff>701040</xdr:colOff>
       <xdr:row>44</xdr:row>
       <xdr:rowOff>121</xdr:rowOff>
     </xdr:to>
@@ -1957,7 +1954,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>702945</xdr:colOff>
+      <xdr:colOff>706755</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>2086</xdr:rowOff>
     </xdr:to>
@@ -2001,9 +1998,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>705277</xdr:colOff>
+      <xdr:colOff>701467</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>288608</xdr:rowOff>
+      <xdr:rowOff>284798</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2045,7 +2042,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>705802</xdr:colOff>
+      <xdr:colOff>701992</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>2527</xdr:rowOff>
     </xdr:to>
@@ -2091,7 +2088,7 @@
       <xdr:col>12</xdr:col>
       <xdr:colOff>689085</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>284798</xdr:rowOff>
+      <xdr:rowOff>288608</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2133,7 +2130,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>705803</xdr:colOff>
+      <xdr:colOff>701993</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>184</xdr:rowOff>
     </xdr:to>
@@ -2177,9 +2174,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>705276</xdr:colOff>
+      <xdr:colOff>701466</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>283366</xdr:rowOff>
+      <xdr:rowOff>287176</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2221,7 +2218,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>707707</xdr:colOff>
+      <xdr:colOff>703897</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>121</xdr:rowOff>
     </xdr:to>
@@ -2309,7 +2306,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>707707</xdr:colOff>
+      <xdr:colOff>703897</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>304921</xdr:rowOff>
     </xdr:to>
@@ -2353,9 +2350,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>701045</xdr:colOff>
+      <xdr:colOff>704855</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>289526</xdr:rowOff>
+      <xdr:rowOff>285716</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2397,9 +2394,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>665797</xdr:colOff>
+      <xdr:colOff>669607</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>287963</xdr:rowOff>
+      <xdr:rowOff>284153</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2441,9 +2438,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>286762</xdr:colOff>
+      <xdr:colOff>282952</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>1921204</xdr:rowOff>
+      <xdr:rowOff>1925014</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3148,7 +3145,7 @@
       <c r="D26" s="47"/>
       <c r="E26" s="45"/>
       <c r="F26" s="82" t="s">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="G26" s="106" t="s">
         <v>134</v>
@@ -3252,7 +3249,7 @@
       </c>
       <c r="C31" s="15" t="str">
         <f>F26</f>
-        <v>LMT_55</v>
+        <v>Pharmed</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="16" t="e">
@@ -3959,36 +3956,36 @@
       <c r="J19" s="86"/>
     </row>
     <row r="20" spans="1:10" s="28" customFormat="1" ht="30.45" customHeight="1">
-      <c r="A20" s="125" t="s">
+      <c r="A20" s="139" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="129" t="s">
+      <c r="B20" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="130"/>
-      <c r="D20" s="130"/>
-      <c r="E20" s="131"/>
+      <c r="C20" s="126"/>
+      <c r="D20" s="126"/>
+      <c r="E20" s="127"/>
       <c r="F20" s="108" t="s">
         <v>45</v>
       </c>
-      <c r="G20" s="135" t="s">
+      <c r="G20" s="131" t="s">
         <v>46</v>
       </c>
-      <c r="H20" s="136"/>
-      <c r="I20" s="139" t="s">
+      <c r="H20" s="132"/>
+      <c r="I20" s="135" t="s">
         <v>53</v>
       </c>
-      <c r="J20" s="140"/>
+      <c r="J20" s="136"/>
     </row>
     <row r="21" spans="1:10" s="28" customFormat="1" ht="21" customHeight="1">
-      <c r="A21" s="125"/>
-      <c r="B21" s="132"/>
-      <c r="C21" s="133"/>
-      <c r="D21" s="133"/>
-      <c r="E21" s="134"/>
+      <c r="A21" s="139"/>
+      <c r="B21" s="128"/>
+      <c r="C21" s="129"/>
+      <c r="D21" s="129"/>
+      <c r="E21" s="130"/>
       <c r="F21" s="108"/>
-      <c r="G21" s="137"/>
-      <c r="H21" s="138"/>
+      <c r="G21" s="133"/>
+      <c r="H21" s="134"/>
       <c r="I21" s="43" t="s">
         <v>47</v>
       </c>
@@ -4000,17 +3997,17 @@
       <c r="A22" s="30">
         <v>1</v>
       </c>
-      <c r="B22" s="122" t="s">
+      <c r="B22" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="123"/>
-      <c r="D22" s="123"/>
-      <c r="E22" s="124"/>
+      <c r="C22" s="120"/>
+      <c r="D22" s="120"/>
+      <c r="E22" s="121"/>
       <c r="F22" s="32"/>
-      <c r="G22" s="120" t="s">
+      <c r="G22" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H22" s="121"/>
+      <c r="H22" s="138"/>
       <c r="I22" s="33"/>
       <c r="J22" s="92"/>
     </row>
@@ -4018,17 +4015,17 @@
       <c r="A23" s="32">
         <v>2</v>
       </c>
-      <c r="B23" s="122" t="s">
+      <c r="B23" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="123"/>
-      <c r="D23" s="123"/>
-      <c r="E23" s="124"/>
+      <c r="C23" s="120"/>
+      <c r="D23" s="120"/>
+      <c r="E23" s="121"/>
       <c r="F23" s="35"/>
-      <c r="G23" s="120" t="s">
+      <c r="G23" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H23" s="121"/>
+      <c r="H23" s="138"/>
       <c r="I23" s="35"/>
       <c r="J23" s="93"/>
     </row>
@@ -4036,17 +4033,17 @@
       <c r="A24" s="32">
         <v>3</v>
       </c>
-      <c r="B24" s="122" t="s">
+      <c r="B24" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="123"/>
-      <c r="D24" s="123"/>
-      <c r="E24" s="124"/>
+      <c r="C24" s="120"/>
+      <c r="D24" s="120"/>
+      <c r="E24" s="121"/>
       <c r="F24" s="35"/>
-      <c r="G24" s="120" t="s">
+      <c r="G24" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="121"/>
+      <c r="H24" s="138"/>
       <c r="I24" s="35"/>
       <c r="J24" s="93"/>
     </row>
@@ -4054,17 +4051,17 @@
       <c r="A25" s="32">
         <v>4</v>
       </c>
-      <c r="B25" s="122" t="s">
+      <c r="B25" s="119" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="123"/>
-      <c r="D25" s="123"/>
-      <c r="E25" s="124"/>
+      <c r="C25" s="120"/>
+      <c r="D25" s="120"/>
+      <c r="E25" s="121"/>
       <c r="F25" s="36"/>
-      <c r="G25" s="120" t="s">
+      <c r="G25" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="121"/>
+      <c r="H25" s="138"/>
       <c r="I25" s="35"/>
       <c r="J25" s="93"/>
     </row>
@@ -4072,17 +4069,17 @@
       <c r="A26" s="32">
         <v>5</v>
       </c>
-      <c r="B26" s="122" t="s">
+      <c r="B26" s="119" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="123"/>
-      <c r="D26" s="123"/>
-      <c r="E26" s="124"/>
+      <c r="C26" s="120"/>
+      <c r="D26" s="120"/>
+      <c r="E26" s="121"/>
       <c r="F26" s="37"/>
-      <c r="G26" s="120" t="s">
+      <c r="G26" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H26" s="121"/>
+      <c r="H26" s="138"/>
       <c r="I26" s="35"/>
       <c r="J26" s="93"/>
     </row>
@@ -4090,17 +4087,17 @@
       <c r="A27" s="32">
         <v>6</v>
       </c>
-      <c r="B27" s="122" t="s">
+      <c r="B27" s="119" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="123"/>
-      <c r="D27" s="123"/>
-      <c r="E27" s="124"/>
+      <c r="C27" s="120"/>
+      <c r="D27" s="120"/>
+      <c r="E27" s="121"/>
       <c r="F27" s="37"/>
-      <c r="G27" s="120" t="s">
+      <c r="G27" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H27" s="121"/>
+      <c r="H27" s="138"/>
       <c r="I27" s="35"/>
       <c r="J27" s="93"/>
     </row>
@@ -4108,17 +4105,17 @@
       <c r="A28" s="32">
         <v>7</v>
       </c>
-      <c r="B28" s="122" t="s">
+      <c r="B28" s="119" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="123"/>
-      <c r="D28" s="123"/>
-      <c r="E28" s="124"/>
+      <c r="C28" s="120"/>
+      <c r="D28" s="120"/>
+      <c r="E28" s="121"/>
       <c r="F28" s="37"/>
-      <c r="G28" s="120" t="s">
+      <c r="G28" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H28" s="121"/>
+      <c r="H28" s="138"/>
       <c r="I28" s="35"/>
       <c r="J28" s="93"/>
     </row>
@@ -4126,17 +4123,17 @@
       <c r="A29" s="37">
         <v>8</v>
       </c>
-      <c r="B29" s="122" t="s">
+      <c r="B29" s="119" t="s">
         <v>43</v>
       </c>
-      <c r="C29" s="123"/>
-      <c r="D29" s="123"/>
-      <c r="E29" s="124"/>
+      <c r="C29" s="120"/>
+      <c r="D29" s="120"/>
+      <c r="E29" s="121"/>
       <c r="F29" s="31"/>
-      <c r="G29" s="120" t="s">
+      <c r="G29" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H29" s="121"/>
+      <c r="H29" s="138"/>
       <c r="I29" s="35"/>
       <c r="J29" s="93"/>
     </row>
@@ -4144,17 +4141,17 @@
       <c r="A30" s="37">
         <v>9</v>
       </c>
-      <c r="B30" s="122" t="s">
+      <c r="B30" s="119" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="123"/>
-      <c r="D30" s="123"/>
-      <c r="E30" s="124"/>
+      <c r="C30" s="120"/>
+      <c r="D30" s="120"/>
+      <c r="E30" s="121"/>
       <c r="F30" s="31"/>
-      <c r="G30" s="120" t="s">
+      <c r="G30" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H30" s="121"/>
+      <c r="H30" s="138"/>
       <c r="I30" s="35"/>
       <c r="J30" s="93"/>
     </row>
@@ -4162,17 +4159,17 @@
       <c r="A31" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="126" t="s">
+      <c r="B31" s="122" t="s">
         <v>12</v>
       </c>
-      <c r="C31" s="127"/>
-      <c r="D31" s="127"/>
-      <c r="E31" s="128"/>
+      <c r="C31" s="123"/>
+      <c r="D31" s="123"/>
+      <c r="E31" s="124"/>
       <c r="F31" s="31"/>
-      <c r="G31" s="120" t="s">
+      <c r="G31" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="H31" s="121"/>
+      <c r="H31" s="138"/>
       <c r="I31" s="35"/>
       <c r="J31" s="93"/>
     </row>
@@ -4225,21 +4222,21 @@
       <c r="J35" s="86"/>
     </row>
     <row r="36" spans="1:13" s="28" customFormat="1" ht="21" customHeight="1">
-      <c r="A36" s="119" t="s">
+      <c r="A36" s="140" t="s">
         <v>64</v>
       </c>
-      <c r="B36" s="119"/>
-      <c r="C36" s="119"/>
-      <c r="D36" s="119"/>
-      <c r="E36" s="119"/>
-      <c r="F36" s="119"/>
-      <c r="G36" s="119"/>
-      <c r="H36" s="119"/>
-      <c r="I36" s="119"/>
-      <c r="J36" s="119"/>
-      <c r="K36" s="119"/>
-      <c r="L36" s="119"/>
-      <c r="M36" s="119"/>
+      <c r="B36" s="140"/>
+      <c r="C36" s="140"/>
+      <c r="D36" s="140"/>
+      <c r="E36" s="140"/>
+      <c r="F36" s="140"/>
+      <c r="G36" s="140"/>
+      <c r="H36" s="140"/>
+      <c r="I36" s="140"/>
+      <c r="J36" s="140"/>
+      <c r="K36" s="140"/>
+      <c r="L36" s="140"/>
+      <c r="M36" s="140"/>
     </row>
     <row r="37" spans="1:13" s="28" customFormat="1" ht="40.950000000000003" customHeight="1">
       <c r="A37" s="72" t="s">
@@ -4293,7 +4290,7 @@
         <v>2.72</v>
       </c>
       <c r="D38" s="73" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="E38" s="103"/>
       <c r="F38" s="103"/>
@@ -4356,7 +4353,9 @@
       <c r="C40" s="73">
         <v>2.84</v>
       </c>
-      <c r="D40" s="73"/>
+      <c r="D40" s="73" t="s">
+        <v>125</v>
+      </c>
       <c r="E40" s="103"/>
       <c r="F40" s="104"/>
       <c r="G40" s="73">
@@ -4450,7 +4449,9 @@
         <v>3.45</v>
       </c>
       <c r="D43" s="73"/>
-      <c r="E43" s="104"/>
+      <c r="E43" s="104" t="s">
+        <v>121</v>
+      </c>
       <c r="F43" s="105"/>
       <c r="G43" s="73">
         <v>152</v>
@@ -4482,7 +4483,9 @@
       </c>
       <c r="D44" s="73"/>
       <c r="E44" s="103"/>
-      <c r="F44" s="103"/>
+      <c r="F44" s="103" t="s">
+        <v>128</v>
+      </c>
       <c r="G44" s="73">
         <v>152</v>
       </c>
@@ -4551,19 +4554,6 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B20:E21"/>
-    <mergeCell ref="G20:H21"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="A1:J5"/>
-    <mergeCell ref="B22:E22"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="H36:M36"/>
     <mergeCell ref="G30:H30"/>
@@ -4580,6 +4570,19 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:E28"/>
     <mergeCell ref="B29:E29"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="A1:J5"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B20:E21"/>
+    <mergeCell ref="G20:H21"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="B23:E23"/>
   </mergeCells>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.51181102362204722" right="0.11811023622047245" top="0.35433070866141736" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -4590,7 +4593,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FF915FA9-662F-4BBC-ACDC-22805800E086}">
           <x14:formula1>
-            <xm:f>INDIRECT('A1'!F26)</xm:f>
+            <xm:f>INDIRECT('A1'!$F$26)</xm:f>
           </x14:formula1>
           <xm:sqref>D38:F45</xm:sqref>
         </x14:dataValidation>

</xml_diff>

<commit_message>
final version of the application without UI design
</commit_message>
<xml_diff>
--- a/examples/TAAT/ใบสั่งงาน TAAT.xlsx
+++ b/examples/TAAT/ใบสั่งงาน TAAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vatska\software\examples\TAAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17C9108-E61C-4C85-A699-1E624C8B9206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B46D464-DBF4-401F-B0AD-D9D540CC8AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{874D8AF1-DF56-4DEE-86B1-A5E2F5D42D71}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="136">
   <si>
     <r>
       <t>บริษัท แวตสก้า จำกัด/ Vatska Company Limited</t>
@@ -489,7 +489,7 @@
     <t>What if " LMT55, Pharmed or E3603" then show dropdown list" worksheet A2, column D,E,F -line 38-48</t>
   </si>
   <si>
-    <t>LMT_55</t>
+    <t>A053404-EP-CP</t>
   </si>
 </sst>
 </file>
@@ -1739,7 +1739,7 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>685804</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>324768</xdr:rowOff>
+      <xdr:rowOff>320958</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1781,7 +1781,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>701040</xdr:colOff>
+      <xdr:colOff>704850</xdr:colOff>
       <xdr:row>42</xdr:row>
       <xdr:rowOff>932</xdr:rowOff>
     </xdr:to>
@@ -1825,9 +1825,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>708133</xdr:colOff>
+      <xdr:colOff>704323</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>286703</xdr:rowOff>
+      <xdr:rowOff>282893</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1869,9 +1869,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>701992</xdr:colOff>
+      <xdr:colOff>705802</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>287839</xdr:rowOff>
+      <xdr:rowOff>284029</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1913,7 +1913,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>704850</xdr:colOff>
+      <xdr:colOff>701040</xdr:colOff>
       <xdr:row>44</xdr:row>
       <xdr:rowOff>121</xdr:rowOff>
     </xdr:to>
@@ -1957,7 +1957,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>702945</xdr:colOff>
+      <xdr:colOff>706755</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>2086</xdr:rowOff>
     </xdr:to>
@@ -2001,9 +2001,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>705277</xdr:colOff>
+      <xdr:colOff>701467</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>288608</xdr:rowOff>
+      <xdr:rowOff>284798</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2045,7 +2045,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>705802</xdr:colOff>
+      <xdr:colOff>701992</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>2527</xdr:rowOff>
     </xdr:to>
@@ -2091,7 +2091,7 @@
       <xdr:col>12</xdr:col>
       <xdr:colOff>689085</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>284798</xdr:rowOff>
+      <xdr:rowOff>288608</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2133,7 +2133,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>705803</xdr:colOff>
+      <xdr:colOff>701993</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>184</xdr:rowOff>
     </xdr:to>
@@ -2177,9 +2177,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>705276</xdr:colOff>
+      <xdr:colOff>701466</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>283366</xdr:rowOff>
+      <xdr:rowOff>287176</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2221,7 +2221,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>707707</xdr:colOff>
+      <xdr:colOff>703897</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>121</xdr:rowOff>
     </xdr:to>
@@ -2309,7 +2309,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>707707</xdr:colOff>
+      <xdr:colOff>703897</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>304921</xdr:rowOff>
     </xdr:to>
@@ -2353,9 +2353,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>701045</xdr:colOff>
+      <xdr:colOff>704855</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>289526</xdr:rowOff>
+      <xdr:rowOff>285716</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2397,9 +2397,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>665797</xdr:colOff>
+      <xdr:colOff>669607</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>287963</xdr:rowOff>
+      <xdr:rowOff>284153</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2441,9 +2441,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>286762</xdr:colOff>
+      <xdr:colOff>282952</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>1921204</xdr:rowOff>
+      <xdr:rowOff>1925014</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2908,7 +2908,9 @@
       <c r="A11" s="44" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="69"/>
+      <c r="B11" s="69" t="s">
+        <v>135</v>
+      </c>
       <c r="C11" s="85"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
@@ -3148,7 +3150,7 @@
       <c r="D26" s="47"/>
       <c r="E26" s="45"/>
       <c r="F26" s="82" t="s">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="G26" s="106" t="s">
         <v>134</v>
@@ -3252,7 +3254,7 @@
       </c>
       <c r="C31" s="15" t="str">
         <f>F26</f>
-        <v>LMT_55</v>
+        <v>Pharmed</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="16" t="e">
@@ -4293,7 +4295,7 @@
         <v>2.72</v>
       </c>
       <c r="D38" s="73" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="E38" s="103"/>
       <c r="F38" s="103"/>
@@ -4356,7 +4358,9 @@
       <c r="C40" s="73">
         <v>2.84</v>
       </c>
-      <c r="D40" s="73"/>
+      <c r="D40" s="73" t="s">
+        <v>125</v>
+      </c>
       <c r="E40" s="103"/>
       <c r="F40" s="104"/>
       <c r="G40" s="73">
@@ -4450,7 +4454,9 @@
         <v>3.45</v>
       </c>
       <c r="D43" s="73"/>
-      <c r="E43" s="104"/>
+      <c r="E43" s="104" t="s">
+        <v>121</v>
+      </c>
       <c r="F43" s="105"/>
       <c r="G43" s="73">
         <v>152</v>
@@ -4482,7 +4488,9 @@
       </c>
       <c r="D44" s="73"/>
       <c r="E44" s="103"/>
-      <c r="F44" s="103"/>
+      <c r="F44" s="103" t="s">
+        <v>128</v>
+      </c>
       <c r="G44" s="73">
         <v>152</v>
       </c>
@@ -4590,7 +4598,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FF915FA9-662F-4BBC-ACDC-22805800E086}">
           <x14:formula1>
-            <xm:f>INDIRECT('A1'!F26)</xm:f>
+            <xm:f>INDIRECT('A1'!$F$26)</xm:f>
           </x14:formula1>
           <xm:sqref>D38:F45</xm:sqref>
         </x14:dataValidation>

</xml_diff>

<commit_message>
final version w/0 design
</commit_message>
<xml_diff>
--- a/examples/TAAT/ใบสั่งงาน TAAT.xlsx
+++ b/examples/TAAT/ใบสั่งงาน TAAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vatska\software\examples\TAAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17C9108-E61C-4C85-A699-1E624C8B9206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B46D464-DBF4-401F-B0AD-D9D540CC8AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{874D8AF1-DF56-4DEE-86B1-A5E2F5D42D71}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="136">
   <si>
     <r>
       <t>บริษัท แวตสก้า จำกัด/ Vatska Company Limited</t>
@@ -489,7 +489,7 @@
     <t>What if " LMT55, Pharmed or E3603" then show dropdown list" worksheet A2, column D,E,F -line 38-48</t>
   </si>
   <si>
-    <t>LMT_55</t>
+    <t>A053404-EP-CP</t>
   </si>
 </sst>
 </file>
@@ -1739,7 +1739,7 @@
       <xdr:col>9</xdr:col>
       <xdr:colOff>685804</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>324768</xdr:rowOff>
+      <xdr:rowOff>320958</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1781,7 +1781,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>701040</xdr:colOff>
+      <xdr:colOff>704850</xdr:colOff>
       <xdr:row>42</xdr:row>
       <xdr:rowOff>932</xdr:rowOff>
     </xdr:to>
@@ -1825,9 +1825,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>708133</xdr:colOff>
+      <xdr:colOff>704323</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>286703</xdr:rowOff>
+      <xdr:rowOff>282893</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1869,9 +1869,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>701992</xdr:colOff>
+      <xdr:colOff>705802</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>287839</xdr:rowOff>
+      <xdr:rowOff>284029</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1913,7 +1913,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>704850</xdr:colOff>
+      <xdr:colOff>701040</xdr:colOff>
       <xdr:row>44</xdr:row>
       <xdr:rowOff>121</xdr:rowOff>
     </xdr:to>
@@ -1957,7 +1957,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>702945</xdr:colOff>
+      <xdr:colOff>706755</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>2086</xdr:rowOff>
     </xdr:to>
@@ -2001,9 +2001,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>705277</xdr:colOff>
+      <xdr:colOff>701467</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>288608</xdr:rowOff>
+      <xdr:rowOff>284798</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2045,7 +2045,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>705802</xdr:colOff>
+      <xdr:colOff>701992</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>2527</xdr:rowOff>
     </xdr:to>
@@ -2091,7 +2091,7 @@
       <xdr:col>12</xdr:col>
       <xdr:colOff>689085</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>284798</xdr:rowOff>
+      <xdr:rowOff>288608</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2133,7 +2133,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>705803</xdr:colOff>
+      <xdr:colOff>701993</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>184</xdr:rowOff>
     </xdr:to>
@@ -2177,9 +2177,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>705276</xdr:colOff>
+      <xdr:colOff>701466</xdr:colOff>
       <xdr:row>38</xdr:row>
-      <xdr:rowOff>283366</xdr:rowOff>
+      <xdr:rowOff>287176</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2221,7 +2221,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>707707</xdr:colOff>
+      <xdr:colOff>703897</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>121</xdr:rowOff>
     </xdr:to>
@@ -2309,7 +2309,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>707707</xdr:colOff>
+      <xdr:colOff>703897</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>304921</xdr:rowOff>
     </xdr:to>
@@ -2353,9 +2353,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>701045</xdr:colOff>
+      <xdr:colOff>704855</xdr:colOff>
       <xdr:row>44</xdr:row>
-      <xdr:rowOff>289526</xdr:rowOff>
+      <xdr:rowOff>285716</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2397,9 +2397,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>665797</xdr:colOff>
+      <xdr:colOff>669607</xdr:colOff>
       <xdr:row>40</xdr:row>
-      <xdr:rowOff>287963</xdr:rowOff>
+      <xdr:rowOff>284153</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2441,9 +2441,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>286762</xdr:colOff>
+      <xdr:colOff>282952</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>1921204</xdr:rowOff>
+      <xdr:rowOff>1925014</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2908,7 +2908,9 @@
       <c r="A11" s="44" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="69"/>
+      <c r="B11" s="69" t="s">
+        <v>135</v>
+      </c>
       <c r="C11" s="85"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
@@ -3148,7 +3150,7 @@
       <c r="D26" s="47"/>
       <c r="E26" s="45"/>
       <c r="F26" s="82" t="s">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="G26" s="106" t="s">
         <v>134</v>
@@ -3252,7 +3254,7 @@
       </c>
       <c r="C31" s="15" t="str">
         <f>F26</f>
-        <v>LMT_55</v>
+        <v>Pharmed</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="16" t="e">
@@ -4293,7 +4295,7 @@
         <v>2.72</v>
       </c>
       <c r="D38" s="73" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="E38" s="103"/>
       <c r="F38" s="103"/>
@@ -4356,7 +4358,9 @@
       <c r="C40" s="73">
         <v>2.84</v>
       </c>
-      <c r="D40" s="73"/>
+      <c r="D40" s="73" t="s">
+        <v>125</v>
+      </c>
       <c r="E40" s="103"/>
       <c r="F40" s="104"/>
       <c r="G40" s="73">
@@ -4450,7 +4454,9 @@
         <v>3.45</v>
       </c>
       <c r="D43" s="73"/>
-      <c r="E43" s="104"/>
+      <c r="E43" s="104" t="s">
+        <v>121</v>
+      </c>
       <c r="F43" s="105"/>
       <c r="G43" s="73">
         <v>152</v>
@@ -4482,7 +4488,9 @@
       </c>
       <c r="D44" s="73"/>
       <c r="E44" s="103"/>
-      <c r="F44" s="103"/>
+      <c r="F44" s="103" t="s">
+        <v>128</v>
+      </c>
       <c r="G44" s="73">
         <v>152</v>
       </c>
@@ -4590,7 +4598,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FF915FA9-662F-4BBC-ACDC-22805800E086}">
           <x14:formula1>
-            <xm:f>INDIRECT('A1'!F26)</xm:f>
+            <xm:f>INDIRECT('A1'!$F$26)</xm:f>
           </x14:formula1>
           <xm:sqref>D38:F45</xm:sqref>
         </x14:dataValidation>

</xml_diff>